<commit_message>
Drop training/sim and ground-transport rows from flight spreadsheet
Keeps only actual flights (operated and passenger positioning); removes
the simulator/training and car-transfer entries.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flights'!$A$1:$E$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flights'!$A$1:$E$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,7 +49,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -131,9 +126,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -513,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -580,71 +572,71 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CAR1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>789</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Ground transport (car)</t>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CAR1</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>332/333</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Ground transport (car)</t>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -652,21 +644,21 @@
           <t>789</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IE19</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -676,24 +668,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>332</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Training / Sim</t>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>IE19</t>
+          <t>60</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HND</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -703,51 +695,51 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>333</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Training / Sim</t>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IE29</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>IE29</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -757,61 +749,61 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
+          <t>388</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>JL86</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>HND</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>332/333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Passenger (positioning)</t>
+          <t>Passenger — Japan Airlines</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>789</t>
+          <t>332</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -823,93 +815,93 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>125</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EF39</t>
+          <t>126</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>IE39</t>
+          <t>127</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IE39</t>
+          <t>128</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -919,24 +911,24 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>292</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HND</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -949,70 +941,70 @@
           <t>333</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>CX360</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>330</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>CX362</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>388</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>JL86</t>
+          <t>CX365</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1022,7 +1014,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>HND</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1030,102 +1022,102 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Japan Airlines</t>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>CX367</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>CX368</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>CX376</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>CX377</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1135,51 +1127,51 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>333</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>CX381</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>HKG</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>333</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>418</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1189,7 +1181,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1201,223 +1193,223 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CX360</t>
+          <t>427</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CX362</t>
+          <t>428</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CX365</t>
+          <t>440</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CX367</t>
+          <t>441</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CX368</t>
+          <t>442</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CX376</t>
+          <t>443</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CX377</t>
+          <t>445</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CX381</t>
+          <t>447</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>448</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1444,7 +1436,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1471,7 +1463,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>458</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1498,7 +1490,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>462</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1525,17 +1517,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>474</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1543,16 +1535,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>442</t>
+          <t>486</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1570,26 +1562,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>443</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1597,16 +1589,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>502</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1616,7 +1608,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1633,17 +1625,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>447</t>
+          <t>505</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1660,12 +1652,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>507</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1687,7 +1679,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>455</t>
+          <t>508</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1697,7 +1689,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1714,17 +1706,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1741,12 +1733,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1768,17 +1760,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>512</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1795,12 +1787,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>486</t>
+          <t>517</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1813,26 +1805,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>520</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1849,17 +1841,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>525</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1876,17 +1868,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>505</t>
+          <t>526</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1903,7 +1895,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>507</t>
+          <t>527</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1921,16 +1913,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>528</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -1957,17 +1949,17 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>529</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1975,26 +1967,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>532</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2011,17 +2003,17 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>533</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2038,7 +2030,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>517</t>
+          <t>535</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2053,7 +2045,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -2065,7 +2057,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>536</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2083,16 +2075,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>525</t>
+          <t>539</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2119,7 +2111,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>526</t>
+          <t>540</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2146,7 +2138,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>541</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2164,16 +2156,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>544</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2200,7 +2192,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>529</t>
+          <t>545</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2218,26 +2210,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>551</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2254,7 +2246,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>555</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2281,22 +2273,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>535</t>
+          <t>604</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -2308,12 +2300,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>536</t>
+          <t>608</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2326,26 +2318,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>610</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2362,17 +2354,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>611</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2389,17 +2381,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>612</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2416,17 +2408,17 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>544</t>
+          <t>613</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2443,7 +2435,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>545</t>
+          <t>615</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2453,7 +2445,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2470,17 +2462,17 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>616</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2497,7 +2489,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>617</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2507,7 +2499,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2524,7 +2516,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>604</t>
+          <t>618</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2542,16 +2534,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>620</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2578,7 +2570,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>622</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2605,7 +2597,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>611</t>
+          <t>625</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2632,7 +2624,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>612</t>
+          <t>626</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2659,7 +2651,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>613</t>
+          <t>627</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2686,17 +2678,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>615</t>
+          <t>628</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2713,17 +2705,17 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>616</t>
+          <t>629</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2740,7 +2732,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>617</t>
+          <t>631</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2767,7 +2759,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>632</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2785,26 +2777,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>633</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -2821,7 +2813,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>634</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2848,7 +2840,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>625</t>
+          <t>637</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -2866,26 +2858,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>626</t>
+          <t>649</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -2893,26 +2885,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>627</t>
+          <t>652</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -2929,17 +2921,17 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>628</t>
+          <t>670</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2947,21 +2939,21 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E90" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>629</t>
+          <t>672</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -2974,26 +2966,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>631</t>
+          <t>673</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3001,16 +2993,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>632</t>
+          <t>685</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -3020,7 +3012,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3028,21 +3020,21 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>633</t>
+          <t>690</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -3055,16 +3047,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E94" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>634</t>
+          <t>693</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3074,7 +3066,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3082,21 +3074,21 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E95" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>694</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -3109,7 +3101,7 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E96" s="5" t="inlineStr">
+      <c r="E96" s="4" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3118,17 +3110,17 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>649</t>
+          <t>695</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3136,26 +3128,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>696</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3163,53 +3155,53 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>670</t>
+          <t>697</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
           <t>ADL</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
           <t>73H</t>
         </is>
       </c>
-      <c r="E99" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>707</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -3217,26 +3209,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>673</t>
+          <t>708</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -3244,26 +3236,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>685</t>
+          <t>712</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -3271,7 +3263,7 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E102" s="5" t="inlineStr">
+      <c r="E102" s="4" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3280,17 +3272,17 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>690</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -3298,26 +3290,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>717</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -3325,34 +3317,34 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>694</t>
+          <t>735</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
           <t>ADL</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
           <t>73H</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E105" s="4" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3361,12 +3353,12 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>695</t>
+          <t>743</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -3379,16 +3371,16 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>696</t>
+          <t>744</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -3398,7 +3390,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -3406,7 +3398,7 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E107" s="5" t="inlineStr">
+      <c r="E107" s="4" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3415,44 +3407,44 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>697</t>
+          <t>760</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E108" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -3460,26 +3452,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>708</t>
+          <t>770</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -3496,25 +3488,25 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>712</t>
+          <t>773</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
+          <t>332</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3523,17 +3515,17 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>884</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -3541,26 +3533,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>717</t>
+          <t>889</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -3568,26 +3560,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>932</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -3595,26 +3587,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>937</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -3622,26 +3614,26 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E115" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>940</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -3649,85 +3641,85 @@
           <t>73H</t>
         </is>
       </c>
-      <c r="E116" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>760</t>
+          <t>1254</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>1257</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E118" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>1881</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
@@ -3739,103 +3731,103 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>773</t>
+          <t>1884</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="E120" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>E90</t>
+        </is>
+      </c>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>884</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E121" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>E90</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>889</t>
+          <t>7301</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E122" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>932</t>
+          <t>7301</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E123" s="3" t="inlineStr">
@@ -3847,7 +3839,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>937</t>
+          <t>7306</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3857,39 +3849,39 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E124" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+          <t>32X</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>940</t>
+          <t>7309</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
           <t>PER</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E125" s="3" t="inlineStr">
@@ -3901,12 +3893,12 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>1254</t>
+          <t>7313</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -3916,7 +3908,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
@@ -3928,22 +3920,22 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>1257</t>
+          <t>7318</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="E127" s="3" t="inlineStr">
@@ -3955,22 +3947,22 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>1881</t>
+          <t>7318</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>E90</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
@@ -3982,12 +3974,12 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>1884</t>
+          <t>7321</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>TSV</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -3997,34 +3989,34 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="E129" s="7" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
+          <t>32X</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Operated</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>7331</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>E90</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -4036,22 +4028,22 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>7301</t>
+          <t>7332</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>TSV</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
@@ -4063,22 +4055,22 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>7301</t>
+          <t>7334</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
@@ -4090,7 +4082,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>7306</t>
+          <t>7335</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -4117,22 +4109,22 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>7309</t>
+          <t>7340</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -4144,22 +4136,22 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>7313</t>
+          <t>7345</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
@@ -4171,22 +4163,22 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>7318</t>
+          <t>7345</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
@@ -4198,22 +4190,22 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>7318</t>
+          <t>7350</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
@@ -4225,17 +4217,17 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>7321</t>
+          <t>7351</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -4252,17 +4244,17 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>7331</t>
+          <t>7353</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4279,17 +4271,17 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>7332</t>
+          <t>7354</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -4306,17 +4298,17 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>7334</t>
+          <t>7356</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4333,22 +4325,22 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>7335</t>
+          <t>7359</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
@@ -4360,22 +4352,22 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>7340</t>
+          <t>7365</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E143" s="3" t="inlineStr">
@@ -4387,22 +4379,22 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>7367</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>HBA</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
@@ -4414,22 +4406,22 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>7376</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>HBA</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
@@ -4441,17 +4433,17 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>7350</t>
+          <t>7390</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -4468,22 +4460,22 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>7351</t>
+          <t>7396</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
@@ -4495,17 +4487,17 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>7353</t>
+          <t>7398</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -4522,17 +4514,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>7354</t>
+          <t>7523</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -4549,22 +4541,22 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>7356</t>
+          <t>7523</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
@@ -4576,22 +4568,22 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>7359</t>
+          <t>7524</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
@@ -4603,17 +4595,17 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>7365</t>
+          <t>7524</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -4630,22 +4622,22 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>7367</t>
+          <t>7525</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E153" s="3" t="inlineStr">
@@ -4657,22 +4649,22 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>7376</t>
+          <t>7526</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
@@ -4684,7 +4676,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>7390</t>
+          <t>7531</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -4694,12 +4686,12 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E155" s="3" t="inlineStr">
@@ -4711,22 +4703,22 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>7396</t>
+          <t>7532</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
@@ -4738,22 +4730,22 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>7398</t>
+          <t>7533</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
@@ -4765,22 +4757,22 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>7534</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
@@ -4792,7 +4784,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>7535</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -4802,12 +4794,12 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E159" s="3" t="inlineStr">
@@ -4819,22 +4811,22 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>7536</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
@@ -4846,12 +4838,12 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>7536</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -4861,7 +4853,7 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="E161" s="3" t="inlineStr">
@@ -4870,251 +4862,8 @@
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" s="2" t="inlineStr">
-        <is>
-          <t>7525</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E162" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
-        <is>
-          <t>7526</t>
-        </is>
-      </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E163" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
-        <is>
-          <t>7531</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E164" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
-        <is>
-          <t>7532</t>
-        </is>
-      </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E165" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
-        <is>
-          <t>7533</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E166" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>7534</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E167" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>7535</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E168" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E169" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="E170" s="3" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E170"/>
+  <autoFilter ref="A1:E161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5125,7 +4874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5133,156 +4882,144 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Qantas A330 crew roster — flight numbers &amp; routes</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr"/>
+      <c r="B1" s="8" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>48 Bid-Period (BP) roster files in the Roster/ folder</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Extracted from</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>'Pattern Details' section of each roster (Depart / Arrive ports)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Rows</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>169 distinct flight + route combinations</t>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>160 distinct flight + route combinations</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Training/simulator and ground (car) positioning — flights only</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Type legend</t>
-        </is>
-      </c>
+      <c r="A6" s="9" t="inlineStr"/>
       <c r="B6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Operated</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
+          <t>Type legend</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Operated</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Flight operated by the crew member (QF)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Deadhead / positioning as a passenger on a QF flight</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Number appears both operated and positioning across rosters</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Positioning on a Cathay Pacific (CX) service</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Passenger — Japan Airlines</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Positioning on a Japan Airlines (JL) service</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Training / Sim</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Simulator/ground training (departure = destination); not an actual flight</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Ground transport (car)</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Positioning by road (CAR); not an actual flight</t>
-        </is>
-      </c>
+      <c r="A13" s="9" t="inlineStr"/>
+      <c r="B13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Some flight numbers appear with more than one route (multi-sector or reused numbers); each route is its own row.</t>
         </is>

</xml_diff>

<commit_message>
Add published scheduled departure/arrival times to flight spreadsheet
Adds Sched Dep and Sched Arr columns (local times) sourced from public
flight-schedule sites via web search, not the roster's actual times.
140 of 160 flight-routes have published times; 20 freighter/WSI/partner
legs marked n/a. Notes tab documents sources and caveats.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated'!$A$1:$E$125</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated'!$A$1:$G$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
@@ -51,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DEEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -110,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -124,13 +135,16 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,7 +153,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -507,14 +521,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,10 +551,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Sched Dep (local)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sched Arr (local)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Aircraft</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
@@ -562,10 +588,20 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>388</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -589,10 +625,20 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>789</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -616,10 +662,20 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>330</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -643,10 +699,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>07:25 +1</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>388</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -670,10 +736,20 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -697,10 +773,20 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>00:45 +1</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -724,10 +810,20 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -751,10 +847,20 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>333</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -778,10 +884,20 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>07:55 +1</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>333</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -805,10 +921,20 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>07:25 +1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>333</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -832,10 +958,20 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -859,10 +995,20 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -886,10 +1032,20 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -913,10 +1069,20 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -940,10 +1106,20 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -967,10 +1143,20 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -994,10 +1180,20 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1021,10 +1217,20 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1048,10 +1254,20 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1075,10 +1291,20 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1102,10 +1328,20 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1129,10 +1365,20 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1156,10 +1402,20 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -1183,10 +1439,20 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1210,10 +1476,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1237,10 +1513,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
+          <t>06:05</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1264,10 +1550,20 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1291,10 +1587,20 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1318,10 +1624,20 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1345,10 +1661,20 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1372,10 +1698,20 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1399,10 +1735,20 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1426,10 +1772,20 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1453,10 +1809,20 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1480,10 +1846,20 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1507,10 +1883,20 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1534,10 +1920,20 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1561,10 +1957,20 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1588,10 +1994,20 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1615,10 +2031,20 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1642,10 +2068,20 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1669,10 +2105,20 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1696,10 +2142,20 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1723,10 +2179,20 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1750,10 +2216,20 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1777,10 +2253,20 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1804,10 +2290,20 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1831,10 +2327,20 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1858,10 +2364,20 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1885,10 +2401,20 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1912,10 +2438,20 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1939,10 +2475,20 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1966,10 +2512,20 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -1993,10 +2549,20 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2020,10 +2586,20 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2047,10 +2623,20 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -2074,10 +2660,20 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2101,10 +2697,20 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2128,10 +2734,20 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2155,10 +2771,20 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2182,10 +2808,20 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2209,10 +2845,20 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2236,10 +2882,20 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2263,10 +2919,20 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2290,10 +2956,20 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2317,10 +2993,20 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2344,10 +3030,20 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2371,10 +3067,20 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -2398,10 +3104,20 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2425,10 +3141,20 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -2452,10 +3178,20 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2479,10 +3215,20 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="inlineStr">
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2506,10 +3252,20 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2533,10 +3289,20 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2560,10 +3326,20 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2587,10 +3363,20 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2614,10 +3400,20 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2641,10 +3437,20 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -2668,10 +3474,20 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>00:25 +1</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2695,10 +3511,20 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
           <t>223</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="G81" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2722,10 +3548,20 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
           <t>223</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
+      <c r="G82" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2749,10 +3585,20 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
           <t>E90</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr">
+      <c r="G83" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2776,10 +3622,20 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
           <t>E90</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>Operated; Passenger (positioning)</t>
         </is>
@@ -2803,10 +3659,20 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
           <t>E90</t>
         </is>
       </c>
-      <c r="E85" s="3" t="inlineStr">
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2828,12 +3694,22 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E86" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2855,12 +3731,22 @@
           <t>WSI</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E87" s="3" t="inlineStr">
+      <c r="G87" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2882,12 +3768,22 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr">
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2909,12 +3805,22 @@
           <t>PER</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E89" s="3" t="inlineStr">
+      <c r="G89" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2938,10 +3844,20 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>21:13</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E90" s="3" t="inlineStr">
+      <c r="G90" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2963,12 +3879,22 @@
           <t>SYD</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr">
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -2990,12 +3916,22 @@
           <t>WSI</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr">
+      <c r="G92" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3017,12 +3953,22 @@
           <t>CNS</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr">
+      <c r="G93" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3044,12 +3990,22 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E94" s="3" t="inlineStr">
+      <c r="G94" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3073,10 +4029,20 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
+          <t>04:35</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E95" s="3" t="inlineStr">
+      <c r="G95" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3100,10 +4066,20 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>00:30 +1</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="G96" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3127,10 +4103,20 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>00:35 +1</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E97" s="3" t="inlineStr">
+      <c r="G97" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3152,12 +4138,22 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="E98" s="3" t="inlineStr">
+      <c r="G98" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3181,10 +4177,20 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>23:50</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E99" s="3" t="inlineStr">
+      <c r="G99" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3206,12 +4212,22 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E100" s="3" t="inlineStr">
+      <c r="G100" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3233,12 +4249,22 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E101" s="3" t="inlineStr">
+      <c r="G101" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3260,12 +4286,22 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E102" s="3" t="inlineStr">
+      <c r="G102" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3289,10 +4325,20 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
+          <t>01:18</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>02:21</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E103" s="3" t="inlineStr">
+      <c r="G103" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3316,10 +4362,20 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E104" s="3" t="inlineStr">
+      <c r="G104" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3343,10 +4399,20 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E105" s="3" t="inlineStr">
+      <c r="G105" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3370,10 +4436,20 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E106" s="3" t="inlineStr">
+      <c r="G106" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3397,10 +4473,20 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E107" s="3" t="inlineStr">
+      <c r="G107" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3424,10 +4510,20 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E108" s="3" t="inlineStr">
+      <c r="G108" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3451,10 +4547,20 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E109" s="3" t="inlineStr">
+      <c r="G109" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3476,12 +4582,22 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E110" s="3" t="inlineStr">
+      <c r="G110" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3503,12 +4619,22 @@
           <t>PER</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="E111" s="3" t="inlineStr">
+      <c r="G111" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3530,12 +4656,22 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E112" s="3" t="inlineStr">
+      <c r="G112" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3559,10 +4695,20 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
+          <t>04:10</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>05:25</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E113" s="3" t="inlineStr">
+      <c r="G113" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3586,10 +4732,20 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>02:10 +1</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="E114" s="3" t="inlineStr">
+      <c r="G114" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3611,12 +4767,22 @@
           <t>SYD</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
         <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E115" s="3" t="inlineStr">
+      <c r="G115" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3640,10 +4806,20 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
+          <t>06:25</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
           <t>32X</t>
         </is>
       </c>
-      <c r="E116" s="3" t="inlineStr">
+      <c r="G116" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3667,10 +4843,20 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E117" s="3" t="inlineStr">
+      <c r="G117" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3694,10 +4880,20 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>09:05 +1</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E118" s="3" t="inlineStr">
+      <c r="G118" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3721,10 +4917,20 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E119" s="3" t="inlineStr">
+      <c r="G119" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3746,12 +4952,22 @@
           <t>HKG</t>
         </is>
       </c>
-      <c r="D120" s="2" t="inlineStr">
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E120" s="3" t="inlineStr">
+      <c r="G120" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3773,12 +4989,22 @@
           <t>PVG</t>
         </is>
       </c>
-      <c r="D121" s="2" t="inlineStr">
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E121" s="3" t="inlineStr">
+      <c r="G121" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3802,10 +5028,20 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E122" s="3" t="inlineStr">
+      <c r="G122" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3827,12 +5063,22 @@
           <t>PVG</t>
         </is>
       </c>
-      <c r="D123" s="2" t="inlineStr">
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E123" s="3" t="inlineStr">
+      <c r="G123" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3856,10 +5102,20 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E124" s="3" t="inlineStr">
+      <c r="G124" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
@@ -3883,17 +5139,27 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="E125" s="3" t="inlineStr">
+      <c r="G125" s="3" t="inlineStr">
         <is>
           <t>Operated</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E125"/>
+  <autoFilter ref="A1:G125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3904,14 +5170,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3932,10 +5200,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Sched Dep (local)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sched Arr (local)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Aircraft</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
@@ -3959,10 +5237,20 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>789</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -3986,10 +5274,20 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>07:50 +1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>332/333</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4013,10 +5311,20 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>08:50 +1</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4040,10 +5348,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>08:55 +1</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>333</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4065,12 +5383,22 @@
           <t>HND</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Passenger — Japan Airlines</t>
         </is>
@@ -4094,10 +5422,20 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4121,10 +5459,20 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4148,10 +5496,20 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4175,10 +5533,20 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4202,10 +5570,20 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4229,10 +5607,20 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4256,10 +5644,20 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4283,10 +5681,20 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -4310,10 +5718,20 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4337,10 +5755,20 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4364,10 +5792,20 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4391,10 +5829,20 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4418,10 +5866,20 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4445,10 +5903,20 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4472,10 +5940,20 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
+          <t>05:35</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4499,10 +5977,20 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4526,10 +6014,20 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
+          <t>06:25</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4553,10 +6051,20 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4580,10 +6088,20 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4607,10 +6125,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4634,10 +6162,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4661,10 +6199,20 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4688,10 +6236,20 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4715,10 +6273,20 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4742,10 +6310,20 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4769,10 +6347,20 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4796,10 +6384,20 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4823,10 +6421,20 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4850,10 +6458,20 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
           <t>332</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4877,10 +6495,20 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
@@ -4904,17 +6532,27 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E37"/>
+  <autoFilter ref="A1:G37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4925,178 +6563,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Qantas A330 crew roster — flight numbers &amp; routes</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr"/>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Qantas A330 crew roster — flights, routes &amp; scheduled times</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Source (flights &amp; routes)</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>48 Bid-Period (BP) roster files in the Roster/ folder</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Extracted from</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>'Pattern Details' section of each roster (Depart / Arrive ports)</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Source (scheduled times)</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Public flight-schedule sources via web search (FlightAware/Airportia/Flightmapper etc.)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Training/simulator and ground (car) positioning — flights only</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Important</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled times are the airlines' PUBLISHED timetable times — NOT the actual times in the roster files.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr"/>
-      <c r="B5" s="9" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Times shown</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Local clock time at each airport (24h). '+1' = arrives next day.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
+          <t>n/a entries</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Qantas Freight A330F services and not-yet-open Western Sydney (WSI) routes have no public passenger timetable; JAL leg not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Caveats</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Times vary by day/season; where sources differed the most common value was taken. Verify against Qantas for a specific date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
           <t>Tabs</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>124 rows — flights operated by the crew (incl. numbers that also appear as positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Positioning</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>36 rows — deadhead / passenger travel (QF, Cathay Pacific, Japan Airlines)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr"/>
       <c r="B9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Type legend</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr"/>
+          <t>Operated</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>124 rows — flights operated by the crew (QF)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Operated</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Flight operated by the crew member (QF)</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Positioning</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>36 rows — deadhead / passenger travel (QF, Cathay Pacific CX, Japan Airlines JL)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Deadhead / positioning as a passenger on a QF flight</t>
-        </is>
-      </c>
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Operated; Passenger (positioning)</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Number appears both operated and positioning across rosters</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Positioning on a Cathay Pacific (CX) service</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Passenger — Japan Airlines</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Positioning on a Japan Airlines (JL) service</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Some flight numbers appear with more than one route (multi-sector or reused numbers); each route is its own row.</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>140 of 160 rows have published scheduled times; 20 marked n/a.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove 7318 PER-SYD row
Operated (freighter) tab now 39 rows; flight 7318 retains only PER-WSI.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$G$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$G$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -787,17 +787,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7318</t>
+          <t>7321</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>TSV</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -824,17 +824,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7321</t>
+          <t>7331</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>7331</t>
+          <t>7332</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>TSV</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>04:35</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>06:40</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7332</t>
+          <t>7334</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -908,17 +908,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>04:35</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>00:30 +1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>7334</t>
+          <t>7335</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -945,17 +945,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:15</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>00:30 +1</t>
+          <t>00:35 +1</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -972,32 +972,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>7335</t>
+          <t>7340</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>22:15</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>00:35 +1</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1009,7 +1009,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>7340</t>
+          <t>7345</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1019,22 +1019,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>23:50</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1059,14 +1059,14 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>22:25</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>23:50</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>7350</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1120,7 +1120,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>7350</t>
+          <t>7351</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>7351</t>
+          <t>7353</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1170,14 +1170,14 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>01:18</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>02:21</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1194,7 +1194,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>7353</t>
+          <t>7354</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1204,17 +1204,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>02:21</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1231,7 +1231,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>7354</t>
+          <t>7356</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1241,17 +1241,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1268,7 +1268,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>7356</t>
+          <t>7359</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1278,22 +1278,22 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>01:30</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1305,32 +1305,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>7359</t>
+          <t>7365</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1342,7 +1342,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>7365</t>
+          <t>7367</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1352,17 +1352,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>HBA</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1379,27 +1379,27 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>7367</t>
+          <t>7376</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>HBA</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>LST</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>HBA</t>
-        </is>
-      </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1416,27 +1416,27 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>7376</t>
+          <t>7390</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>20:30</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1453,19 +1453,19 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>7390</t>
+          <t>7396</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>PER</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1490,17 +1490,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>7396</t>
+          <t>7398</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1527,27 +1527,27 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>7398</t>
+          <t>7523</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>04:10</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>05:25</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1569,27 +1569,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>AKL</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>CHC</t>
-        </is>
-      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>04:10</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>05:25</t>
+          <t>02:10 +1</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1601,32 +1601,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>7524</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>21:10</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>02:10 +1</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1651,14 +1651,14 @@
           <t>SYD</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>06:25</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>07:40</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1675,32 +1675,32 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>7525</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>06:25</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1712,27 +1712,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>7525</t>
+          <t>7526</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>09:05 +1</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1749,27 +1749,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>7526</t>
+          <t>7531</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
           <t>HKG</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>09:05 +1</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>7531</t>
+          <t>7532</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1799,14 +1799,14 @@
           <t>HKG</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>12:15</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>19:45</t>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1823,17 +1823,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>7532</t>
+          <t>7533</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1860,27 +1860,27 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>7533</t>
+          <t>7534</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>18:20</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1897,27 +1897,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>7534</t>
+          <t>7535</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
           <t>PVG</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>04:45</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>18:20</t>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1934,27 +1934,27 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>7535</t>
+          <t>7536</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>07:49</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1976,22 +1976,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>02:45</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2005,45 +2005,8 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>03:30</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G41"/>
+  <autoFilter ref="A1:G40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6650,7 +6613,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>40 rows — QF7XXX A330 freighter services flown by the crew</t>
+          <t>39 rows — QF7XXX A330 freighter services flown by the crew</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove 7345 SYD-MEL and 7301 SYD-BNE rows
Operated (freighter) tab now 37 rows; 7345 retains WSI-MEL, 7301 retains SYD-WSI.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$G$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -602,17 +602,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>7301</t>
+          <t>7306</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -639,17 +639,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>7306</t>
+          <t>7309</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -676,27 +676,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>7309</t>
+          <t>7313</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>21:13</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -713,32 +713,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>7313</t>
+          <t>7318</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>19:18</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>21:13</t>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -750,17 +750,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>7318</t>
+          <t>7321</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>TSV</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -787,17 +787,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7321</t>
+          <t>7331</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7331</t>
+          <t>7332</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -834,17 +834,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>TSV</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>04:35</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>06:40</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>7332</t>
+          <t>7334</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>04:35</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>00:30 +1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7334</t>
+          <t>7335</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -908,17 +908,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:15</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>00:30 +1</t>
+          <t>00:35 +1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -935,32 +935,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>7335</t>
+          <t>7340</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>22:15</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>00:35 +1</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -972,17 +972,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>7340</t>
+          <t>7345</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1009,32 +1009,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>7350</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>22:25</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>23:50</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1046,17 +1046,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>7351</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1083,7 +1083,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>7350</t>
+          <t>7353</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1096,14 +1096,14 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>01:18</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>02:21</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1120,7 +1120,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>7351</t>
+          <t>7354</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1130,17 +1130,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>21:25</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>7353</t>
+          <t>7356</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1167,17 +1167,17 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>02:21</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1194,7 +1194,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>7354</t>
+          <t>7359</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1204,22 +1204,22 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>01:30</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1231,27 +1231,27 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>7356</t>
+          <t>7365</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1268,32 +1268,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>7359</t>
+          <t>7367</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>HBA</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1305,27 +1305,27 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>7365</t>
+          <t>7376</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
+          <t>HBA</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
           <t>LST</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1342,27 +1342,27 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>7367</t>
+          <t>7390</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>03:30</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>04:00</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1379,32 +1379,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>7376</t>
+          <t>7396</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>20:30</t>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>7390</t>
+          <t>7398</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1453,32 +1453,32 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>7396</t>
+          <t>7523</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>04:10</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>05:25</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1490,32 +1490,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>7398</t>
+          <t>7523</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>AKL</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>02:10 +1</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>32X/33X</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>7524</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1537,17 +1537,17 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>04:10</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>05:25</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1564,32 +1564,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>7524</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>06:25</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>02:10 +1</t>
+          <t>07:40</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
+          <t>32X</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1601,32 +1601,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>7525</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>18:45</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1638,12 +1638,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>7526</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1653,17 +1653,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>06:25</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>09:05 +1</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1675,12 +1675,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>7525</t>
+          <t>7531</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1712,27 +1712,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>7526</t>
+          <t>7532</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>HKG</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>09:05 +1</t>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1749,27 +1749,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>7531</t>
+          <t>7533</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>12:15</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>19:45</t>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1786,27 +1786,27 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>7532</t>
+          <t>7534</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>18:20</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1823,7 +1823,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>7533</t>
+          <t>7535</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1860,7 +1860,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>7534</t>
+          <t>7536</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>02:45</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1897,27 +1897,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>7535</t>
+          <t>7536</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1931,82 +1931,8 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>02:45</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>07:49</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>03:30</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G40"/>
+  <autoFilter ref="A1:G38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6613,7 +6539,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>39 rows — QF7XXX A330 freighter services flown by the crew</t>
+          <t>37 rows — QF7XXX A330 freighter services flown by the crew</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add user-supplied WSI freighter times for 7301 and 7318
7301 SYD-WSI 12:30->13:15; 7318 PER-WSI 13:50->19:50 (local).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -71,12 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -124,11 +124,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -578,14 +578,14 @@
           <t>WSI</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -615,12 +615,12 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -630,7 +630,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -652,12 +652,12 @@
           <t>PER</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -667,7 +667,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -704,7 +704,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -726,14 +726,14 @@
           <t>WSI</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -763,12 +763,12 @@
           <t>CNS</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -778,7 +778,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -800,12 +800,12 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -815,7 +815,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -852,7 +852,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -889,7 +889,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -926,7 +926,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -948,12 +948,12 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -963,7 +963,7 @@
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -985,12 +985,12 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1000,7 +1000,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1022,12 +1022,12 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1037,7 +1037,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1059,12 +1059,12 @@
           <t>BNE</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1074,7 +1074,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1111,7 +1111,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1148,7 +1148,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1185,7 +1185,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1222,7 +1222,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1259,7 +1259,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1296,7 +1296,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1333,7 +1333,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1355,12 +1355,12 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1370,7 +1370,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1392,12 +1392,12 @@
           <t>PER</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1407,7 +1407,7 @@
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1429,12 +1429,12 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1444,7 +1444,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1481,7 +1481,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1518,7 +1518,7 @@
           <t>32X/33X</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1540,12 +1540,12 @@
           <t>SYD</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1555,7 +1555,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1592,7 +1592,7 @@
           <t>32X</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1629,7 +1629,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1666,7 +1666,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1703,7 +1703,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1725,12 +1725,12 @@
           <t>HKG</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1740,7 +1740,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1762,12 +1762,12 @@
           <t>PVG</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1777,7 +1777,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1814,7 +1814,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1836,12 +1836,12 @@
           <t>PVG</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1851,7 +1851,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1888,7 +1888,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -1925,7 +1925,7 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Operated (freighter)</t>
         </is>
@@ -2304,12 +2304,12 @@
           <t>HND</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Public flight-schedule sources via web search (FlightAware/Airportia/Flightmapper etc.)</t>
+          <t>Public flight-schedule sources via web search; WSI freighter times supplied by user.</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Airlines' PUBLISHED timetable times (local clock, 24h; '+1' = next day) — NOT the actual times in the roster files.</t>
+          <t>PUBLISHED timetable times (local clock, 24h; '+1' = next day) — NOT the actual times in the roster files.</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Most QF7XXX freighter services and not-yet-open Western Sydney (WSI) routes have no public timetable; JAL leg times not found.</t>
+          <t>Remaining QF7XXX freighter services with no public timetable; JAL leg times not found.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild freighter tab from official Qantas Freight timetable
Operated (freighter) tab now transcribed directly from the supplied
schedule photo: 29 flight-routes with operating Days, STD/STA times,
Aircraft (A330/A321) and Network (Domestic/International). Freighter
flights not in the photo removed; 7305 and 7330 added. Positioning tab
unchanged (120 rows).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$G$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,11 +51,6 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -76,12 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -124,14 +119,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -143,9 +141,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -513,16 +508,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,29 +539,34 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Sched Dep (local)</t>
+          <t>Days</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Sched Arr (local)</t>
+          <t>STD (dep)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>STA (arr)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Aircraft</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Network</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>7301</t>
+          <t>QF7301</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -578,36 +579,41 @@
           <t>WSI</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>13:15</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>7306</t>
+          <t>QF7345</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -615,31 +621,36 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>7309</t>
+          <t>QF7359</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -652,179 +663,204 @@
           <t>PER</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>7313</t>
+          <t>QF7318</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>19:18</t>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Thu</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>7318</t>
+          <t>QF7313</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>13:50</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>7321</t>
+          <t>QF7335</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>TSV</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>22:20</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7331</t>
+          <t>QF7353</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>01:40</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>03:55</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7332</t>
+          <t>QF7332</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -837,253 +873,288 @@
           <t>TSV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>04:35</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>04:50</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>7334</t>
+          <t>QF7321</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>TSV</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>22:00</t>
+          <t>CNS</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>00:30 +1</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7335</t>
+          <t>QF7376</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>HBA</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>22:15</t>
+          <t>LST</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>00:35 +1</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>7340</t>
+          <t>QF7365</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>21:00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>7345</t>
+          <t>QF7350</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>23:00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>7350</t>
+          <t>QF7305</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>02:10</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>04:35</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>7351</t>
+          <t>QF7398</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>19:15</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>7353</t>
+          <t>QF7356</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1093,71 +1164,81 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>01:18</t>
+          <t>LST</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>02:21</t>
+          <t>02:25</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>7354</t>
+          <t>QF7367</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>20:05</t>
+          <t>HBA</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>04:25</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>04:55</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>7356</t>
+          <t>QF7354</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1167,76 +1248,86 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>02:30</t>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>7359</t>
+          <t>QF7340</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>01:30</t>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>22:25</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>00:05</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>7365</t>
+          <t>QF7330</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1244,695 +1335,454 @@
           <t>MEL</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>21:00</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>03:25</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>7367</t>
+          <t>QF7390</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>03:30</t>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>03:50</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Domestic</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>7376</t>
+          <t>QF7525</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HBA</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>LST</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Wed, Sun</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>7390</t>
+          <t>QF7526</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Wed, Fri, Sun</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>23:45</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>7396</t>
+          <t>QF7531</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>7398</t>
+          <t>QF7535</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Thu, Sat</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>00:20</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>QF7536</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>04:10</t>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Wed, Sun</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>05:25</t>
+          <t>02:40</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>7523</t>
+          <t>QF7536</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>AKL</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>21:10</t>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Wed, Sun</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>02:10 +1</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>32X/33X</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>A330</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>QF7523</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
           <t>AKL</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Mon–Thu, Sat</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>22:10</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>03:10</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>7524</t>
+          <t>QF7523</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>AKL</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>CHC</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>06:25</t>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri, Sun</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>04:10</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>32X</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>05:25</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>7525</t>
+          <t>QF7524</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>12:15</t>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Tue–Fri, Sun</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>06:25</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>7526</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>09:05 +1</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>7531</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>12:15</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>7532</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>HKG</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>7533</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>7534</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>04:45</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>18:20</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>7535</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>PVG</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>02:45</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>07:49</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>7536</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>03:30</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>A321</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G38"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2304,12 +2154,12 @@
           <t>HND</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2319,7 +2169,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Passenger — Japan Airlines</t>
         </is>
@@ -2578,7 +2428,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2615,7 +2465,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2652,7 +2502,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2689,7 +2539,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2726,7 +2576,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2763,7 +2613,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2800,7 +2650,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -2837,7 +2687,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Passenger — Cathay Pacific</t>
         </is>
@@ -6444,114 +6294,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Qantas A330 FREIGHTER crew roster — flights, routes &amp; scheduled times</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr"/>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Qantas A330 crew roster — freighter schedule &amp; positioning</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Source (flights &amp; routes)</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>48 Bid-Period (BP) roster files in the Roster/ folder</t>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Operated (freighter) tab</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Transcribed directly from the official Qantas Freight timetable (photo). All flights, operating days and STD/STA times are from that schedule. Flights not in the photo were removed.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Source (scheduled times)</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Public flight-schedule sources via web search; WSI freighter times supplied by user.</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Operating days per week (Mon–Sun). STD/STA are for the first applicable flight of the week; times vary slightly by day.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Classification</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Crew OPERATE only the QF7XXX A330 freighter services. Every other flight (3-digit QF, QF4/30/38/60, QF1254/1257/1881/1884/1887, Cathay CX, Japan Airlines JL) is POSITIONING / deadhead travel as passengers.</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Aircraft / Network</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Photo groups freighters by A330 vs A321 and Domestic vs International — captured in those columns.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled times</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>PUBLISHED timetable times (local clock, 24h; '+1' = next day) — NOT the actual times in the roster files.</t>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Positioning tab</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Unchanged — deadhead / passenger travel to &amp; from freighter duties (QF, Cathay CX, Japan Airlines JL); scheduled times from public sources.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>n/a entries</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Remaining QF7XXX freighter services with no public timetable; JAL leg times not found.</t>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>International day columns in the photo are small — verify 7525/7526/7531/7535/7536 day patterns if precision matters.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr"/>
-      <c r="B7" s="9" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Tabs</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Operated (freighter)</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>37 rows — QF7XXX A330 freighter services flown by the crew</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Positioning</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>120 rows — deadhead / passenger travel to &amp; from freighter duties</t>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Operated (freighter): 29 rows  |  Positioning: 120 rows</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Patterns tab to spreadsheet
New Patterns sheet lists full flight pairings (OP = operating, PAX =
positioning) with per-day legs, ground times and sign-on/off/rest,
matching the tap-to-view pattern in the app. Seeded with the QF7301/7318
pairing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet name="Operated (freighter)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Positioning" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Patterns" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$K$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,8 +53,18 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +96,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEFEF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -111,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -142,6 +159,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6294,6 +6324,335 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Full flight pairings / patterns — OP = operating, PAX = positioning (deadhead).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Pairing</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Flight</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Dep</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Arr</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Aircraft</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Ground</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>QF7301 pairing</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>10 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>QF7301</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>0:30</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CAR001</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>1:25</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>QF651</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 11:30 · Sign-off 19:25 · Rest 17:25 at PER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>11 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>QF7318</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>0:40</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CAR001</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:50 · Sign-off 21:30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:K7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add QF7345 Monday pairing; make patterns day-aware
Pairings now keyed by flight+weekday (same flight can belong to different
pairings on different days). Adds the QF7345 Monday pairing (WSI-MEL-PER
layover-WSI, incl. block times, rest and TAFB) to both the app pattern
view and the spreadsheet Patterns tab (now with a Blk column).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005B6F95"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -128,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -173,6 +179,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6324,26 +6331,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Full flight pairings / patterns — OP = operating, PAX = positioning (deadhead).</t>
+          <t>Full flight pairings / patterns — OP = operating, PAX = positioning (deadhead). Pairings vary by weekday.</t>
         </is>
       </c>
     </row>
@@ -6395,10 +6403,15 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
+          <t>Blk</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
           <t>Ground</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>Duty</t>
         </is>
@@ -6407,12 +6420,12 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>QF7301 pairing</t>
+          <t>QF7301 pairing · Mon</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>10 Aug 2026</t>
+          <t>10 Aug 2026 (Mon)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -6452,10 +6465,15 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>0:45</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>0:30</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr"/>
+      <c r="L3" s="13" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr"/>
@@ -6495,12 +6513,13 @@
           <t>CAR</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>1:25</t>
         </is>
       </c>
-      <c r="K4" s="13" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr"/>
@@ -6541,7 +6560,8 @@
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="15" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="15" t="inlineStr">
         <is>
           <t>Sign-on 11:30 · Sign-off 19:25 · Rest 17:25 at PER</t>
         </is>
@@ -6551,7 +6571,7 @@
       <c r="A6" s="12" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>11 Aug 2026 (Tue)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -6591,10 +6611,15 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>4:00</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
           <t>0:40</t>
         </is>
       </c>
-      <c r="K6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr"/>
@@ -6635,14 +6660,185 @@
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="15" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="15" t="inlineStr">
         <is>
           <t>Sign-on 12:50 · Sign-off 21:30</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 pairing · Mon</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>10 Aug 2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>QF7359</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Rest 32:30 at PER</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>12 Aug 2026 (Wed)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>QF7318</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>4:00</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:50 · Sign-off 20:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>TAFB 46:15 · Minimum rest 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:K7"/>
+  <autoFilter ref="A2:L12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Show patterns by weekday; add QF7345 Tue/Wed/Thu pairings
Pattern days now labelled by day of week (they repeat weekly) instead of
calendar dates. Adds the QF7345 Tuesday, Wednesday (international via HKG)
and Thursday (positions home) pairings to the app and the spreadsheet
Patterns tab. Handles layover-only duty rows where sign-on/off wasn't shown.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6331,11 +6331,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -6345,13 +6345,13 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Full flight pairings / patterns — OP = operating, PAX = positioning (deadhead). Pairings vary by weekday.</t>
+          <t>Full flight pairings — shown by day of week (they repeat weekly). OP = operating, PAX = positioning.</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -6420,12 +6420,12 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>QF7301 pairing · Mon</t>
+          <t>QF7301 · Mon</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>10 Aug 2026 (Mon)</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -6571,7 +6571,7 @@
       <c r="A6" s="12" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>11 Aug 2026 (Tue)</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -6670,12 +6670,12 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>QF7345 pairing · Mon</t>
+          <t>QF7345 · Mon</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>10 Aug 2026 (Mon)</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -6779,7 +6779,7 @@
       <c r="A11" s="12" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>12 Aug 2026 (Wed)</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -6837,8 +6837,628 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Tue</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>QF7359</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Rest 32:30 at PER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>QF7318</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>4:00</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:50 · Sign-off 20:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Wed</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>QF7359</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>QF7531</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 13:30 · Sign-off 22:15 · Layover at HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>QF7526</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="13" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>CAR001</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="13" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>International pairing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Thu</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>QF7359</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>QF652</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>32Q</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="13" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>CAR001</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>23:55</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="13" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Positions home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L12"/>
+  <autoFilter ref="A2:L29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Drop TAFB/min rest from spreadsheet and app pattern; weekday-only
Removes the TAFB/minimum-rest footer from the Patterns tab and the app
pattern view. Patterns remain labelled by day of week only (no dates).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6331,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6829,25 +6829,67 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>TAFB 46:15 · Minimum rest 15:00</t>
-        </is>
-      </c>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Tue</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>QF7345 · Tue</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
+      <c r="A14" s="12" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="4" t="inlineStr">
         <is>
           <t>OP</t>
@@ -6855,27 +6897,27 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>QF7345</t>
+          <t>QF7359</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>22:50</t>
+          <t>01:55</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>00:25</t>
+          <t>04:05</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -6885,19 +6927,23 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>1:35</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>1:30</t>
-        </is>
-      </c>
-      <c r="L14" s="13" t="inlineStr"/>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Rest 32:30 at PER</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
           <t>OP</t>
@@ -6905,27 +6951,27 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>QF7359</t>
+          <t>QF7318</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>01:55</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>04:05</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -6935,131 +6981,131 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>4:00</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 21:50 · Sign-off 04:20 · Rest 32:30 at PER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
+          <t>Sign-on 12:50 · Sign-off 20:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Wed</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>OP</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>QF7318</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>QF7359</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>01:55</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>PER</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>13:50</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>WSI</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>19:50</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>04:05</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>33X</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>4:00</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 12:50 · Sign-off 20:05</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>QF7345 · Wed</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>QF7345</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>WSI</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>22:50</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>00:25</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>1:35</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>1:30</t>
-        </is>
-      </c>
-      <c r="L18" s="13" t="inlineStr"/>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
           <t>OP</t>
@@ -7067,27 +7113,27 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>QF7359</t>
+          <t>QF7531</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>01:55</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>04:05</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -7095,15 +7141,11 @@
           <t>33X</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
+      <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
+          <t>Sign-on 13:30 · Sign-off 22:15 · Layover at HKG</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7153,7 @@
       <c r="A20" s="12" t="inlineStr"/>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -7121,27 +7163,27 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>QF7531</t>
+          <t>QF7526</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -7151,52 +7193,44 @@
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 13:30 · Sign-off 22:15 · Layover at HKG</t>
-        </is>
-      </c>
+      <c r="L20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>QF7526</t>
+          <t>CAR001</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
@@ -7204,66 +7238,74 @@
       <c r="L21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr"/>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>CAR001</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>International pairing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>QF7345 · Thu</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>QF7345</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>WSI</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>CAR</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="13" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>International pairing</t>
-        </is>
-      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>00:25</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>QF7345 · Thu</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
+      <c r="A25" s="12" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr">
         <is>
           <t>OP</t>
@@ -7271,27 +7313,27 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>QF7345</t>
+          <t>QF7359</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>22:50</t>
+          <t>01:55</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>00:25</t>
+          <t>04:05</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -7301,73 +7343,65 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>1:35</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>1:30</t>
-        </is>
-      </c>
-      <c r="L25" s="13" t="inlineStr"/>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr"/>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>QF7359</t>
+          <t>QF652</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>01:55</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>04:05</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
+          <t>32Q</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 21:50 · Sign-off 04:20 · Layover at PER</t>
-        </is>
-      </c>
+      <c r="L26" s="13" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr"/>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
+      <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="14" t="inlineStr">
         <is>
           <t>PAX</t>
@@ -7375,32 +7409,32 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>QF652</t>
+          <t>CAR001</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:55</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>32Q</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -7408,57 +7442,15 @@
       <c r="L27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>CAR001</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>WSI</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>23:55</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>CAR</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="13" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L29"/>
+  <autoFilter ref="A2:L28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add QF7525 Wednesday pairing (SYD-HKG-SYD)
Adds the 7525 Wed pairing (SYD->HKG Wed, layover, 7526 HKG->SYD Fri) to
the app pattern view and the spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6331,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7449,8 +7449,112 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>QF7525 · Wed</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>QF7525</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 11:20 · Sign-off 20:05 · Layover at HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>QF7526</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 22:40 · Sign-off 11:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L28"/>
+  <autoFilter ref="A2:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add QF7525 Sunday pairing (SYD-HKG-SYD)
Adds the 7525 Sun pairing (SYD->HKG Sun, HKG layover, 7526 HKG->SYD Wed)
to the app pattern view and the spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6331,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7553,8 +7553,108 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>QF7525 · Sun</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>QF7525</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:20 · Sign-off 21:05 · Layover at HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>QF7526</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="13" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L31"/>
+  <autoFilter ref="A2:L34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Z Crew (3rd pilot) pattern variant for QF7535 Thursday
Adds a Normal/Z crew toggle inside the pattern view, shown only when a
Z variant exists. QF7535 Thu now has both: Normal (7535->PVG, 7536->SIN,
pax QF82 home) and Z crew (7535->PVG, pax CX367->HKG, 7526 HKG->SYD).
Both added to the spreadsheet Patterns tab. Flight labels now strip
leading zeros (082 -> QF82).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6331,10 +6331,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -7653,8 +7653,316 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="13" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>QF7535 · Thu</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>QF7535</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>00:20</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>02:40</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 01:40 · Sign-off 08:45 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>QF82</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="13" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Positions home</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>QF7535 · Thu (Z crew)</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>QF7535</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>00:20</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>CX367</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:20 · Sign-off 16:30 · Layover at HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr"/>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>QF7526</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="13" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>3rd crew member</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L34"/>
+  <autoFilter ref="A2:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Spreadsheet: drop positioning flights not originating in Australia
Positioning tab now keeps only flights departing an Australian port
(removes AKL/HKG/HND/PVG/SIN origins) — 103 rows, down from 120.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1830,7 +1830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1919,27 +1919,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>06:45</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>08:20</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1956,32 +1956,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>07:50 +1</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>332/333</t>
+          <t>330</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -1993,32 +1993,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>789</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -2030,32 +2030,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>125</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>AKL</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>08:50 +1</t>
+          <t>00:45 +1</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -2067,27 +2067,27 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>127</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HND</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>08:55 +1</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2104,32 +2104,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>418</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -2141,32 +2141,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>427</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>07:25 +1</t>
+          <t>10:35</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -2178,69 +2178,69 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JL86</t>
+          <t>428</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>HND</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Japan Airlines</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>440</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>13:20</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -2252,27 +2252,27 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>441</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>00:45 +1</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2289,32 +2289,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>442</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>AKL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -2326,7 +2326,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>443</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -2336,22 +2336,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2363,32 +2363,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>445</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>07:55 +1</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -2400,32 +2400,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>447</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>07:25 +1</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2437,308 +2437,308 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CX360</t>
+          <t>448</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CX362</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>22:05</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CX365</t>
+          <t>458</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CX367</t>
+          <t>462</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CX368</t>
+          <t>474</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CX376</t>
+          <t>486</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CX377</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CX381</t>
+          <t>502</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>07:05</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Passenger — Cathay Pacific</t>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Passenger (positioning)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>505</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2748,12 +2748,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>06:05</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2770,27 +2770,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>507</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>10:35</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2807,27 +2807,27 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>508</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2844,27 +2844,27 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2881,27 +2881,27 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2918,27 +2918,27 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>442</t>
+          <t>512</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>10:35</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2955,27 +2955,27 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>443</t>
+          <t>517</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2992,7 +2992,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>520</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3002,17 +3002,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:05</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3029,27 +3029,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>447</t>
+          <t>525</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3066,27 +3066,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>526</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3103,27 +3103,27 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>455</t>
+          <t>527</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3140,27 +3140,27 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>528</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3177,12 +3177,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>529</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3192,12 +3192,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3214,27 +3214,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>532</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3251,12 +3251,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>486</t>
+          <t>533</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3266,12 +3266,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3288,7 +3288,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>535</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3303,17 +3303,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -3325,7 +3325,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>536</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3340,12 +3340,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3362,7 +3362,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>505</t>
+          <t>539</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -3377,12 +3377,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>06:05</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3399,27 +3399,27 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>507</t>
+          <t>540</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -3436,27 +3436,27 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>541</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>08:20</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3473,7 +3473,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>544</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3488,12 +3488,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3510,7 +3510,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>545</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3525,12 +3525,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3547,27 +3547,27 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>551</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
           <t>SYD</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>10:35</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3584,7 +3584,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>517</t>
+          <t>555</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3599,12 +3599,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3621,12 +3621,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>604</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3636,12 +3636,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3658,27 +3658,27 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>525</t>
+          <t>608</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>08:10</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>09:25</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3695,12 +3695,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>526</t>
+          <t>610</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3710,12 +3710,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3732,7 +3732,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>611</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3742,17 +3742,17 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>11:50</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3769,12 +3769,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>612</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3784,12 +3784,12 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3806,7 +3806,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>529</t>
+          <t>613</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -3816,17 +3816,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3843,27 +3843,27 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>615</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3880,27 +3880,27 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>616</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>535</t>
+          <t>617</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3927,22 +3927,22 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>73H</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -3954,12 +3954,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>536</t>
+          <t>618</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3969,12 +3969,12 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3991,27 +3991,27 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>620</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -4028,12 +4028,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>622</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4043,12 +4043,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -4065,7 +4065,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>625</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -4075,17 +4075,17 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -4102,12 +4102,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>544</t>
+          <t>626</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4117,12 +4117,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>545</t>
+          <t>627</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4149,17 +4149,17 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4176,27 +4176,27 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>628</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4213,7 +4213,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>629</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4223,17 +4223,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -4250,27 +4250,27 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>604</t>
+          <t>631</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4287,7 +4287,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>632</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4302,12 +4302,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>08:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>09:25</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -4324,27 +4324,27 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>633</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -4361,27 +4361,27 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>611</t>
+          <t>634</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -4398,27 +4398,27 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>612</t>
+          <t>637</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>22:05</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4435,27 +4435,27 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>613</t>
+          <t>649</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4472,27 +4472,27 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>615</t>
+          <t>652</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4509,27 +4509,27 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>616</t>
+          <t>670</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
+          <t>ADL</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>05:35</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>07:50</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -4546,12 +4546,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>617</t>
+          <t>672</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4561,12 +4561,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>06:35</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4583,7 +4583,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>673</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -4593,17 +4593,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>13:20</t>
+          <t>06:25</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -4620,7 +4620,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>685</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4630,17 +4630,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4657,27 +4657,27 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>690</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>ADL</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -4694,27 +4694,27 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>625</t>
+          <t>693</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -4731,27 +4731,27 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>626</t>
+          <t>694</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
+          <t>ADL</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -4768,27 +4768,27 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>627</t>
+          <t>695</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4805,27 +4805,27 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>628</t>
+          <t>696</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
+          <t>ADL</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -4842,27 +4842,27 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>629</t>
+          <t>697</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4879,27 +4879,27 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>631</t>
+          <t>707</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
+          <t>CNS</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4916,27 +4916,27 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>632</t>
+          <t>708</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4953,7 +4953,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>633</t>
+          <t>712</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4963,17 +4963,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4990,12 +4990,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>634</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -5005,12 +5005,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -5027,27 +5027,27 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>717</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>CNS</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>22:05</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -5064,7 +5064,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>649</t>
+          <t>735</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -5074,17 +5074,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -5101,27 +5101,27 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>743</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -5138,7 +5138,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>670</t>
+          <t>744</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -5148,17 +5148,17 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>05:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>07:50</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -5175,12 +5175,12 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>760</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -5190,17 +5190,17 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>06:35</t>
+          <t>06:15</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5212,7 +5212,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>673</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -5222,17 +5222,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>06:25</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5249,27 +5249,27 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>685</t>
+          <t>770</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>22:25</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -5286,32 +5286,32 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>690</t>
+          <t>773</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -5323,12 +5323,12 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>884</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -5338,12 +5338,12 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -5360,7 +5360,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>694</t>
+          <t>889</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5370,17 +5370,17 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -5397,27 +5397,27 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>695</t>
+          <t>932</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -5434,27 +5434,27 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>696</t>
+          <t>937</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -5471,27 +5471,27 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>697</t>
+          <t>940</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>00:25 +1</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -5508,12 +5508,12 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>1254</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5523,17 +5523,17 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>223</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -5545,7 +5545,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>708</t>
+          <t>1257</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5555,22 +5555,22 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>223</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
@@ -5582,32 +5582,32 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>712</t>
+          <t>1881</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
+          <t>CNS</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr">
@@ -5619,32 +5619,32 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>1884</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
           <t>CNS</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
@@ -5656,7 +5656,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>717</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5671,17 +5671,17 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G104" s="5" t="inlineStr">
@@ -5690,637 +5690,8 @@
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>735</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>11:20</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>743</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>17:40</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>18:50</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>16:25</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>760</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>06:15</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>11:45</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="G108" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>765</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>19:10</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G109" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>770</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>16:55</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>22:25</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G110" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>773</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>13:25</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="G111" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>884</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>889</t>
-        </is>
-      </c>
-      <c r="B113" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>14:50</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>932</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>12:25</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>937</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>940</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>00:25 +1</t>
-        </is>
-      </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G116" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>1254</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t>16:05</t>
-        </is>
-      </c>
-      <c r="E117" s="2" t="inlineStr">
-        <is>
-          <t>18:25</t>
-        </is>
-      </c>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
-      <c r="G117" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>1257</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>15:50</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
-      <c r="G118" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>1881</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>08:20</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G119" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>1884</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>14:25</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G120" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>1887</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G121" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G121"/>
+  <autoFilter ref="A1:G104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7238,7 +6609,6 @@
       <c r="L21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" s="16" t="inlineStr">
         <is>
           <t>International pairing</t>
@@ -7442,7 +6812,6 @@
       <c r="L27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7800,7 +7169,6 @@
       <c r="L38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7954,7 +7322,6 @@
       <c r="L43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" s="16" t="inlineStr">
         <is>
           <t>3rd crew member</t>

</xml_diff>

<commit_message>
Add MEL-crew Wednesday pattern for QF7535 (positioning start)
Surfaces QF470 (MEL->SYD positioning) in MEL + Wednesday results as a
positioning-start entry; tapping it opens the MEL-crew pattern (pos
MEL->SYD, operate 7535 SYD->PVG, 7536 PVG->SIN, pax QF38 SIN->MEL).
Positioning entries render with a Positioning badge, real aircraft type,
and a dashed amber map arc. Added to the spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5702,10 +5702,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -6609,6 +6609,7 @@
       <c r="L21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr"/>
       <c r="B22" s="16" t="inlineStr">
         <is>
           <t>International pairing</t>
@@ -6812,6 +6813,7 @@
       <c r="L27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr"/>
       <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7169,6 +7171,7 @@
       <c r="L38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr"/>
       <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7322,14 +7325,227 @@
       <c r="L43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr"/>
       <c r="B44" s="16" t="inlineStr">
         <is>
           <t>3rd crew member</t>
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>QF7535 · Wed (MEL crew)</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>QF470</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr"/>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>QF7535</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>00:20</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr"/>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>02:40</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 01:40 · Sign-off 08:45 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>QF38</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 22:30 · Sign-off 09:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start from MEL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L44"/>
+  <autoFilter ref="A2:L50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add MEL-crew Thursday pattern (QF7525 via QF470 positioning)
Extends QF470 positioning entry to Thursday for MEL base; tapping it on
Thursday opens the 7525 MEL pattern (pos MEL->SYD, operate 7525 SYD->HKG,
7526 HKG->SYD, pax QF447 home). Added to the spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5702,7 +5702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7544,8 +7544,208 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>QF7525 · Thu (MEL crew)</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>QF470</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>QF7525</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:00 · Sign-off 20:45 · Layover at HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>QF7526</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="13" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>QF447</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>32Q</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="13" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start from MEL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L50"/>
+  <autoFilter ref="A2:L56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add SYD-crew Wednesday pattern (QF7536 via QF127 positioning)
Surfaces QF127 (SYD->HKG positioning) for SYD + Wednesday; tapping opens
the pattern: pos SYD->HKG (QF127) + HKG->PVG (CX362), then operate 7536
PVG->SIN and 7536 SIN->SYD. Added to spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5702,7 +5702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7744,8 +7744,208 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>QF7536 · Wed (SYD crew)</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>QF127</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="13" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr"/>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>CX362</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 09:10 · Sign-off 22:25 · Layover at PVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr"/>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>03:34</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 01:40 · Sign-off 08:50 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr"/>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 10:00 · Sign-off 20:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start via HKG/PVG</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L56"/>
+  <autoFilter ref="A2:L62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add SYD-crew Thursday pattern (QF7536 SIN-SYD via QF81 positioning)
Surfaces QF81 (SYD->SIN positioning) for SYD + Thursday; tapping opens
the pattern: pos SYD->SIN (QF81), then operate 7536 SIN->SYD. Added to
spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5702,7 +5702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7944,8 +7944,120 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>QF7536 · Thu (SYD crew)</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>QF81</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 09:20 · Sign-off 17:25 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 10:00 · Sign-off 20:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start via SIN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L62"/>
+  <autoFilter ref="A2:L66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Spreadsheet: remove positioning flights involving ADL
Positioning tab now excludes any flight with ADL as origin or destination
(15 rows removed); 88 remain.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1830,7 +1830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4509,27 +4509,27 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>670</t>
+          <t>707</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>05:35</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>07:50</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -4546,27 +4546,27 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>708</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>06:35</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4583,27 +4583,27 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>673</t>
+          <t>712</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>06:25</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -4620,27 +4620,27 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>685</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4657,27 +4657,27 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>690</t>
+          <t>717</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -4694,32 +4694,32 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>760</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>06:15</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -4731,27 +4731,27 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>694</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -4768,27 +4768,27 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>695</t>
+          <t>770</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>22:25</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4805,32 +4805,32 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>696</t>
+          <t>773</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>332</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -4842,27 +4842,27 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>697</t>
+          <t>932</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4879,27 +4879,27 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>937</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>PER</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4916,27 +4916,27 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>708</t>
+          <t>940</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>00:25 +1</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4953,32 +4953,32 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>712</t>
+          <t>1254</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>MEL</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
           <t>BNE</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>223</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -4990,32 +4990,32 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>1257</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>223</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>717</t>
+          <t>1881</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -5042,17 +5042,17 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5064,32 +5064,32 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>1884</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5101,32 +5101,32 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>BNE</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>E90</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5135,563 +5135,8 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>16:25</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>760</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>06:15</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>11:45</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>765</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>19:10</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>770</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>16:55</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>22:25</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>773</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>13:25</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>884</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>889</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>ADL</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>14:50</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G96" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>932</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>12:25</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G97" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>937</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>940</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>PER</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>00:25 +1</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>73H</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>1254</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>16:05</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>18:25</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>1257</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>MEL</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>15:50</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>1881</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>08:20</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G102" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>1884</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>14:25</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>1887</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>CNS</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>E90</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>Passenger (positioning)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G104"/>
+  <autoFilter ref="A1:G89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6609,7 +6054,6 @@
       <c r="L21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" s="16" t="inlineStr">
         <is>
           <t>International pairing</t>
@@ -6813,7 +6257,6 @@
       <c r="L27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7171,7 +6614,6 @@
       <c r="L38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -7325,7 +6767,6 @@
       <c r="L43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" s="16" t="inlineStr">
         <is>
           <t>3rd crew member</t>
@@ -7537,7 +6978,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" s="16" t="inlineStr">
         <is>
           <t>Positioning start from MEL</t>
@@ -7737,7 +7177,6 @@
       <c r="L55" s="13" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" s="16" t="inlineStr">
         <is>
           <t>Positioning start from MEL</t>
@@ -7937,7 +7376,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" s="16" t="inlineStr">
         <is>
           <t>Positioning start via HKG/PVG</t>
@@ -8049,7 +7487,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" s="16" t="inlineStr">
         <is>
           <t>Positioning start via SIN</t>

</xml_diff>

<commit_message>
Add QF7535 Saturday pattern (positions home via HKG)
7535 Sat: operate 7535 SYD->PVG, then position PVG->HKG (CX377) and
HKG->SYD (QF128). Added to app and spreadsheet Patterns tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WHSE4rFFukAMEY6xNxZKok
</commit_message>
<xml_diff>
--- a/Roster_Flight_Numbers.xlsx
+++ b/Roster_Flight_Numbers.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operated (freighter)'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Positioning'!$A$1:$G$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Patterns'!$A$2:$L$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5147,7 +5147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6054,6 +6054,7 @@
       <c r="L21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr"/>
       <c r="B22" s="16" t="inlineStr">
         <is>
           <t>International pairing</t>
@@ -6257,6 +6258,7 @@
       <c r="L27" s="13" t="inlineStr"/>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr"/>
       <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -6614,6 +6616,7 @@
       <c r="L38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr"/>
       <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Positions home</t>
@@ -6767,6 +6770,7 @@
       <c r="L43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr"/>
       <c r="B44" s="16" t="inlineStr">
         <is>
           <t>3rd crew member</t>
@@ -6776,54 +6780,54 @@
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>QF7535 · Wed (MEL crew)</t>
+          <t>QF7535 · Sat</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>QF470</t>
+          <t>QF7535</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>00:20</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
+          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
         </is>
       </c>
     </row>
@@ -6831,210 +6835,199 @@
       <c r="A47" s="12" t="inlineStr"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>QF7535</t>
+          <t>CX377</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>00:20</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
-        </is>
-      </c>
+      <c r="L47" s="13" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>QF7536</t>
+          <t>QF128</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>02:40</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>06:45</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>333</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 01:40 · Sign-off 08:45 · Layover at SIN</t>
+          <t>Sign-on 13:30 · Sign-off 07:15</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="inlineStr">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Positions home via HKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>QF7535 · Wed (MEL crew)</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
         <is>
           <t>PAX</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>QF38</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>QF470</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>08:50</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>332</t>
-        </is>
-      </c>
-      <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 22:30 · Sign-off 09:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>Positioning start from MEL</t>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="inlineStr">
-        <is>
-          <t>QF7525 · Thu (MEL crew)</t>
-        </is>
-      </c>
+      <c r="A52" s="12" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>QF470</t>
+          <t>QF7535</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>00:20</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>73H</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
+          <t>Sign-on 14:25 · Sign-off 00:35 · Layover at PVG</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7035,7 @@
       <c r="A53" s="12" t="inlineStr"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -7052,27 +7045,27 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>QF7525</t>
+          <t>QF7536</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>02:40</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -7084,7 +7077,7 @@
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 12:00 · Sign-off 20:45 · Layover at HKG</t>
+          <t>Sign-on 01:40 · Sign-off 08:45 · Layover at SIN</t>
         </is>
       </c>
     </row>
@@ -7095,113 +7088,126 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>QF7526</t>
+          <t>QF38</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>332</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="13" t="inlineStr"/>
+      <c r="L54" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 22:30 · Sign-off 09:20</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr"/>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start from MEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>QF7525 · Thu (MEL crew)</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
         <is>
           <t>PAX</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>QF447</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>QF470</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>15:05</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>32Q</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr"/>
-      <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="13" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="16" t="inlineStr">
-        <is>
-          <t>Positioning start from MEL</t>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>73H</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 16:35 · Sign-off 18:50 · Layover at SYD</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t>QF7536 · Wed (SYD crew)</t>
-        </is>
-      </c>
+      <c r="A58" s="12" t="inlineStr"/>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>QF127</t>
+          <t>QF7525</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -7211,7 +7217,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>10:17</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -7221,29 +7227,37 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>33X</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="13" t="inlineStr"/>
+      <c r="L58" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 12:00 · Sign-off 20:45 · Layover at HKG</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr"/>
-      <c r="B59" s="2" t="inlineStr"/>
-      <c r="C59" s="14" t="inlineStr">
-        <is>
-          <t>PAX</t>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>CX362</t>
+          <t>QF7526</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -7253,146 +7267,131 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>22:10</t>
-        </is>
-      </c>
-      <c r="I59" s="2" t="inlineStr"/>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 09:10 · Sign-off 22:25 · Layover at PVG</t>
-        </is>
-      </c>
+      <c r="L59" s="13" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr"/>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>QF7536</t>
+          <t>QF447</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>PVG</t>
+          <t>SYD</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>03:34</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>MEL</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>08:35</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>33X</t>
+          <t>32Q</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 01:40 · Sign-off 08:50 · Layover at SIN</t>
-        </is>
-      </c>
+      <c r="L60" s="13" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="inlineStr"/>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>OP</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>QF7536</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>SIN</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>10:51</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>20:18</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>33X</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="15" t="inlineStr">
-        <is>
-          <t>Sign-on 10:00 · Sign-off 20:33</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="16" t="inlineStr">
-        <is>
-          <t>Positioning start via HKG/PVG</t>
-        </is>
-      </c>
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start from MEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>QF7536 · Wed (SYD crew)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>QF127</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="13" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>QF7536 · Thu (SYD crew)</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
+      <c r="A64" s="12" t="inlineStr"/>
+      <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="14" t="inlineStr">
         <is>
           <t>PAX</t>
@@ -7400,39 +7399,35 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>QF81</t>
+          <t>CX362</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>SYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>PVG</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>16:55</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>330</t>
-        </is>
-      </c>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="15" t="inlineStr">
         <is>
-          <t>Sign-on 09:20 · Sign-off 17:25 · Layover at SIN</t>
+          <t>Sign-on 09:10 · Sign-off 22:25 · Layover at PVG</t>
         </is>
       </c>
     </row>
@@ -7455,22 +7450,22 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
+          <t>PVG</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>03:34</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
           <t>SIN</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>SYD</t>
-        </is>
-      </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -7482,19 +7477,182 @@
       <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="15" t="inlineStr">
         <is>
+          <t>Sign-on 01:40 · Sign-off 08:50 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr"/>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 10:00 · Sign-off 20:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Positioning start via HKG/PVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>QF7536 · Thu (SYD crew)</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>QF81</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="15" t="inlineStr">
+        <is>
+          <t>Sign-on 09:20 · Sign-off 17:25 · Layover at SIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>QF7536</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>SYD</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>33X</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="15" t="inlineStr">
+        <is>
           <t>Sign-on 10:00 · Sign-off 20:55</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="16" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>Positioning start via SIN</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L66"/>
+  <autoFilter ref="A2:L71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>